<commit_message>
투자 대시보드 2026-09-29 18:25
</commit_message>
<xml_diff>
--- a/technicals/exports/2026-09-28.xlsx
+++ b/technicals/exports/2026-09-28.xlsx
@@ -142,7 +142,7 @@
       </ns0:c>
       <ns0:c r="F2" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계 생명과학, 진단 및 응용화학 시장에 용도별 솔루션을 제공.</ns0:t>
+          <ns0:t>전 세계 생명과학·진단·응용화학 시장에 용도별 솔루션을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G2">
@@ -184,7 +184,7 @@
       </ns0:c>
       <ns0:c r="R2" t="inlineStr">
         <ns0:is>
-          <ns0:t>교환 제안과 반복 매출을 통한 가치평가, 실적 발표 후 9.6% 오른 주가의 지속 가능성이 다뤄졌다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>교환 제안·반복 매출을 둘러싼 기업가치 평가와 최근 실적 발표 이후 주가 9.6% 상승의 지속 가능성 조명. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S2" t="inlineStr">
@@ -226,7 +226,7 @@
       </ns0:c>
       <ns0:c r="F3" t="inlineStr">
         <ns0:is>
-          <ns0:t>미충족 의료 수요에 대응하는 항체 의약품을 개발하며, 비호르몬 치료제 ABCL635는 임상 2상 중.</ns0:t>
+          <ns0:t>미충족 의료 수요에 대응하는 항체 의약품 개발사로, 비호르몬 치료제 ABCL635는 임상 2상 중.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G3">
@@ -268,7 +268,7 @@
       </ns0:c>
       <ns0:c r="R3" t="inlineStr">
         <ns0:is>
-          <ns0:t>ABCL 주가가 3개월간 121% 상승했다는 보도가 나왔다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>애브셀라 주가의 최근 3개월간 121% 상승을 조명. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S3" t="inlineStr">
@@ -310,7 +310,7 @@
       </ns0:c>
       <ns0:c r="F4" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국 뷰티·개인관리 브랜드에 전략, 마케팅, 전 채널 판매, 고객 서비스 및 물류 등 브랜드 관리 제공.</ns0:t>
+          <ns0:t>중국 뷰티·개인관리 브랜드에 전략·마케팅·전 채널 판매·고객 서비스·물류 등 브랜드 관리 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G4">
@@ -386,7 +386,7 @@
       </ns0:c>
       <ns0:c r="F5" t="inlineStr">
         <ns0:is>
-          <ns0:t>북미·아시아태평양 등에서 전문·기술 컨설팅과 운영 모델 설계 관련 자문을 제공.</ns0:t>
+          <ns0:t>북미·아시아태평양 등에서 전문·기술 컨설팅과 운영 모델 설계 자문 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G5">
@@ -507,7 +507,7 @@
       </ns0:c>
       <ns0:c r="R6" t="inlineStr">
         <ns0:is>
-          <ns0:t>임상시험 업데이트와 신규 자금 조달 이후 아제너스 주식의 적정가치 평가가 높아졌다는 보도다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>임상 진행 소식과 신규 자금 조달 이후 아제너스 주식의 적정가치 평가 상향 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S6" t="inlineStr">
@@ -675,7 +675,7 @@
       </ns0:c>
       <ns0:c r="R8" t="inlineStr">
         <ns0:is>
-          <ns0:t>AI 데이터센터 분야에서 앳코어가 주목받는 이유와 전기 시스템 업종 내 우수한 2분기 실적이 다뤄졌다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>AI 데이터센터 관련 기업으로 아트코어가 주목받으며, 전기 시스템 업종 2분기 실적 비교에서 우수 평가. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S8" t="inlineStr">
@@ -717,7 +717,7 @@
       </ns0:c>
       <ns0:c r="F9" t="inlineStr">
         <ns0:is>
-          <ns0:t>자회사를 통해 MLB 애틀랜타 브레이브스 구단과 구장을 소유·운영하며 복합개발 사업을 영위.</ns0:t>
+          <ns0:t>자회사를 통해 MLB 애틀랜타 브레이브스 구단·구장을 소유·운영하고 복합개발 사업 영위.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G9">
@@ -759,7 +759,7 @@
       </ns0:c>
       <ns0:c r="R9" t="inlineStr">
         <ns0:is>
-          <ns0:t>애틀랜타 브레이브스 주주가 가치 실현을 위한 매각과 구단 인수자 물색을 촉구했다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>주주 브리치 인렛이 기업가치 실현을 위한 애틀랜타 브레이브스 매각과 구단 인수자 물색을 촉구. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S9" t="inlineStr">
@@ -801,7 +801,7 @@
       </ns0:c>
       <ns0:c r="F10" t="inlineStr">
         <ns0:is>
-          <ns0:t>자회사를 통해 MLB 애틀랜타 브레이브스 구단과 구장을 소유·운영하며 복합개발 사업을 영위.</ns0:t>
+          <ns0:t>자회사를 통해 MLB 애틀랜타 브레이브스 구단·구장을 소유·운영하고 복합개발 사업 영위.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G10">
@@ -843,7 +843,7 @@
       </ns0:c>
       <ns0:c r="R10" t="inlineStr">
         <ns0:is>
-          <ns0:t>애틀랜타 브레이브스 주주가 가치 실현을 위한 매각과 구단 인수자 물색을 촉구했다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>주주 브리치 인렛이 기업가치 실현을 위한 애틀랜타 브레이브스 매각과 구단 인수자 물색을 촉구. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S10" t="inlineStr">
@@ -885,7 +885,7 @@
       </ns0:c>
       <ns0:c r="F11" t="inlineStr">
         <ns0:is>
-          <ns0:t>폐암 위험 평가를 위한 혈액 기반 폐결절 검사 등 진단 솔루션을 제공.</ns0:t>
+          <ns0:t>폐암 위험 평가를 위한 혈액 기반 폐결절 검사 등 진단 솔루션 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G11">
@@ -927,7 +927,7 @@
       </ns0:c>
       <ns0:c r="R11" t="inlineStr">
         <ns0:is>
-          <ns0:t>종양 정보 활용·비활용 방식으로 MRD 검사를 확대하고 바이오래드·써모피셔와 모니터링 프로그램을 추진했다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>종양 정보 활용·비활용 방식으로 MRD 검사를 확대하고 바이오래드·써모 피셔와 모니터링 프로그램 추진. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S11" t="inlineStr">
@@ -969,7 +969,7 @@
       </ns0:c>
       <ns0:c r="F12" t="inlineStr">
         <ns0:is>
-          <ns0:t>다발성경화증, 척수성 근위축증, 프리드라이히 운동실조증 등의 치료제를 발굴·개발·제조·공급.</ns0:t>
+          <ns0:t>다발성경화증·척수성 근위축증·프리드라이히 운동실조증 등의 치료제를 발굴·개발·제조·공급.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G12">
@@ -1011,7 +1011,7 @@
       </ns0:c>
       <ns0:c r="R12" t="inlineStr">
         <ns0:is>
-          <ns0:t>성장 제품군과 기존 다발성경화증 약물의 실적 비교, 2분기 실적, 가정용 레켐비 펜·신장질환 데이터가 다뤄졌다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>성장 제품군과 기존 다발성경화증 약물의 성과 비교, 2분기 실적, 가정용 레켐비 펜·신장질환 데이터 진전 조명. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S12" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </ns0:c>
       <ns0:c r="R13" t="inlineStr">
         <ns0:is>
-          <ns0:t>다이아몬드힐이 바이오라이프 솔루션스의 높은 전환 비용에 주목해 투자했다는 보도다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>다이아몬드 힐이 바이오라이프 솔루션스의 높은 전환 비용에 주목해 투자. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S13" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </ns0:c>
       <ns0:c r="F14" t="inlineStr">
         <ns0:is>
-          <ns0:t>이식 환자의 치료 결과와 장기 건강 개선을 위한 신장·심장 이식 검사 솔루션 등을 제공하는 기업.</ns0:t>
+          <ns0:t>이식 환자의 치료 결과와 장기 건강 개선을 위한 신장·심장 이식 검사 솔루션 제공 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G14">
@@ -1221,7 +1221,7 @@
       </ns0:c>
       <ns0:c r="F15" t="inlineStr">
         <ns0:is>
-          <ns0:t>자회사와 함께 미국 및 라틴아메리카에서 영화관을 운영하는 영화 상영 기업.</ns0:t>
+          <ns0:t>자회사와 함께 미국·라틴아메리카에서 영화관을 운영하는 영화 상영 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G15">
@@ -1263,7 +1263,7 @@
       </ns0:c>
       <ns0:c r="R15" t="inlineStr">
         <ns0:is>
-          <ns0:t>AMC 주가가 13% 상승한 가운데 시네마크와 아이맥스도 소폭 올랐다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>AMC의 차환 관련 랠리와 13% 상승이 보도된 가운데 시네마크와 IMAX도 소폭 상승. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S15" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </ns0:c>
       <ns0:c r="F16" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 합병, 주식 교환, 자산 인수, 자본 재편 등 기업결합을 추진.</ns0:t>
+          <ns0:t>주요 영업활동 없이 합병·주식 교환·자산 인수·자본 재편 등 기업결합 추진.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G16">
@@ -1381,7 +1381,7 @@
       </ns0:c>
       <ns0:c r="F17" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 기업 합병, 주식 교환, 자산 인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>주요 영업활동 없이 합병·주식 교환·자산 인수 등 기업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G17">
@@ -1460,7 +1460,7 @@
       </ns0:c>
       <ns0:c r="F18" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 소파, 의자, 침실·식당 가구 등 주거용 가구를 제조·유통·수입·판매한다.</ns0:t>
+          <ns0:t>미국에서 소파·의자·침실·식당용 주거 가구를 제조·유통·수입·판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G18">
@@ -1502,7 +1502,7 @@
       </ns0:c>
       <ns0:c r="R18" t="inlineStr">
         <ns0:is>
-          <ns0:t>신고가 경신 후 추가 상승 여력과 올해 경기소비재 업종 대비 주가 성과를 점검하는 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>신고가 경신 후 추가 상승 여력과 올해 경기소비재 종목 대비 수익률을 점검한 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S18" t="inlineStr">
@@ -1544,7 +1544,7 @@
       </ns0:c>
       <ns0:c r="F19" t="inlineStr">
         <ns0:is>
-          <ns0:t>개인과 기업에 예금·은행·자산관리 서비스를 제공하는 퍼스트 시코스트 은행의 지주회사.</ns0:t>
+          <ns0:t>개인·기업에 예금·은행·자산관리 서비스를 제공하는 퍼스트 시코스트 은행의 지주회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G19">
@@ -1620,7 +1620,7 @@
       </ns0:c>
       <ns0:c r="F20" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 캐나다에서 보관·선반, 안전·보안 등 산업용 및 유지보수·수리·운영 제품을 유통한다.</ns0:t>
+          <ns0:t>미국·캐나다에서 보관·선반·안전·보안 등 산업용 및 유지보수·수리·운영 제품을 유통한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G20">
@@ -1662,7 +1662,7 @@
       </ns0:c>
       <ns0:c r="R20" t="inlineStr">
         <ns0:is>
-          <ns0:t>컨퍼런스 참석 이후 기업가치의 주가 반영 여부와 투자 회피 사유를 검토하는 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>컨퍼런스 참석 후 주가의 가치 반영 수준을 점검하고 투자 회피 논거를 제시한 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S20" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </ns0:c>
       <ns0:c r="F21" t="inlineStr">
         <ns0:is>
-          <ns0:t>덴마크 바이오기업으로 암 등 질환 치료용 항체 의약품을 개발하며 EPKINLY·TEPKINLY를 판매한다.</ns0:t>
+          <ns0:t>암 등 질환 치료용 항체 의약품을 개발하고 EPKINLY·TEPKINLY를 판매하는 덴마크 바이오기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G21">
@@ -1788,7 +1788,7 @@
       </ns0:c>
       <ns0:c r="F22" t="inlineStr">
         <ns0:is>
-          <ns0:t>다중암 조기 발견 검사·서비스를 제공하며, 50세 초과 무증상자를 위한 갈레리 암 선별검사를 판매하는 기업.</ns0:t>
+          <ns0:t>다중암 조기 발견 검사·서비스를 제공하고 50세 초과 무증상자용 갈레리 암 선별검사를 판매하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G22">
@@ -1827,7 +1827,7 @@
       </ns0:c>
       <ns0:c r="R22" t="inlineStr">
         <ns0:is>
-          <ns0:t>주간 주가 55% 급등, 암 탐지 혈액검사에 대한 FDA 자문위원 지지, 고평가 여부가 보도됐다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>주간 주가 55% 급등, 암 발견 혈액검사에 대한 FDA 자문위원 지지와 고평가 여부를 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S22" t="inlineStr">
@@ -1869,7 +1869,7 @@
       </ns0:c>
       <ns0:c r="F23" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 기업 합병, 주식 교환, 자산 인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>주요 영업활동 없이 합병·주식 교환·자산 인수 등 기업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G23">
@@ -1945,7 +1945,7 @@
       </ns0:c>
       <ns0:c r="F24" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국과 해외에서 다양한 형태의 맞춤형 냉간 성형 강재를 제조·판매하는 회사.</ns0:t>
+          <ns0:t>중국과 해외에서 다양한 맞춤형 냉간 성형 강재를 제조·판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G24">
@@ -2024,7 +2024,7 @@
       </ns0:c>
       <ns0:c r="F25" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 임원 채용, 산업·건설·사무 인력 공급, 정규직 채용 등 인력 서비스를 제공한다.</ns0:t>
+          <ns0:t>미국에서 임원·정규직 채용과 산업·건설·사무 인력 공급 등 인력 서비스를 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G25">
@@ -2066,7 +2066,7 @@
       </ns0:c>
       <ns0:c r="R25" t="inlineStr">
         <ns0:is>
-          <ns0:t>주가 6.9% 상승과 상승세 지속 가능성을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>주가 6.9% 상승과 추가 상승 가능성을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S25" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </ns0:c>
       <ns0:c r="F26" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다·중화권 등 전 세계에서 엔터테인먼트와 이벤트용 기술 플랫폼을 운영한다.</ns0:t>
+          <ns0:t>미국·캐나다·중화권 등 전 세계에서 엔터테인먼트·이벤트용 기술 플랫폼을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G26">
@@ -2150,7 +2150,7 @@
       </ns0:c>
       <ns0:c r="R26" t="inlineStr">
         <ns0:is>
-          <ns0:t>IMAX 주가 상승과 업종 대비 성과를 점검하고, 모건스탠리의 추가 상승 전망 및 ‘오디세이’의 영향을 조명. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>IMAX 주가 상승과 경기소비재 대비 성과를 점검하고, 모건스탠리의 추가 상승 전망 및 ‘오디세이’ 영향을 소개. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S26" t="inlineStr">
@@ -2234,7 +2234,7 @@
       </ns0:c>
       <ns0:c r="R27" t="inlineStr">
         <ns0:is>
-          <ns0:t>실적 발표 이후 주가 2% 상승과 지속 가능성, 양호한 분기 실적 속 현금흐름 문제가 다뤄졌다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>실적 발표 이후 주가가 2% 오른 가운데, 견조한 분기 실적에 가려진 현금흐름 문제가 지적됐다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S27" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </ns0:c>
       <ns0:c r="F28" t="inlineStr">
         <ns0:is>
-          <ns0:t>자가 종양침윤림프구를 활용해 전이성 흑색종 등 고형암 치료용 세포치료제를 개발·상용화한다.</ns0:t>
+          <ns0:t>자가 종양침윤림프구 기반으로 전이성 흑색종 등 고형암용 세포치료제를 개발·상용화한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G28">
@@ -2318,7 +2318,7 @@
       </ns0:c>
       <ns0:c r="R28" t="inlineStr">
         <ns0:is>
-          <ns0:t>당일 주가 급등의 배경을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>당일 주가 급등 배경을 다룬 기사로, 제목에는 구체적 배경이 제시되지 않음. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S28" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </ns0:c>
       <ns0:c r="F29" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 온·오프라인 채널로 여성 의류·신발·보석·가방 등 액세서리를 판매한다.</ns0:t>
+          <ns0:t>미국 온·오프라인 채널에서 여성 의류·신발·보석·가방 등 액세서리를 판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G29">
@@ -2607,7 +2607,7 @@
       </ns0:c>
       <ns0:c r="F32" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 기업 합병, 주식 교환, 자산 인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>주요 영업활동 없이 합병·주식 교환·자산 인수 등 기업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G32">
@@ -2683,7 +2683,7 @@
       </ns0:c>
       <ns0:c r="F33" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다·영국에서 상장지수상품 운용 서비스를 제공하며 보안시스템·미용제품·금융 사업도 한다.</ns0:t>
+          <ns0:t>미국·캐나다·영국에서 상장지수상품을 운용하며 보안시스템·미용제품·금융 사업도 한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G33">
@@ -2762,7 +2762,7 @@
       </ns0:c>
       <ns0:c r="F34" t="inlineStr">
         <ns0:is>
-          <ns0:t>미주·유럽·아시아 등 전 세계에서 실험실 기기 등 정밀기기를 제조·공급하고 관련 서비스를 제공한다.</ns0:t>
+          <ns0:t>전 세계에서 실험실 기기 등 정밀기기를 제조·공급하고 관련 서비스를 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G34">
@@ -2804,7 +2804,7 @@
       </ns0:c>
       <ns0:c r="R34" t="inlineStr">
         <ns0:is>
-          <ns0:t>메틀러톨레도가 새롭게 주목받는 배경을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>메틀러토레도가 새롭게 주목받는 배경을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S34" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </ns0:c>
       <ns0:c r="F36" t="inlineStr">
         <ns0:is>
-          <ns0:t>분자검사 서비스를 개발·상용화하며 잔존질환 평가·재발 감시·치료 반응 평가용 혈액검사를 제공한다.</ns0:t>
+          <ns0:t>분자검사를 개발·상용화하며 잔존질환·재발 감시·치료 반응 평가용 혈액검사를 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G36">
@@ -2972,7 +2972,7 @@
       </ns0:c>
       <ns0:c r="R36" t="inlineStr">
         <ns0:is>
-          <ns0:t>시그나테라의 방광암 동반진단 일본 PMDA 승인과 주가 급등이 보도됐다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>시그나테라가 일본 PMDA의 방광암 동반진단 승인을 받았으며, 주가 급등을 다룬 기사도 나왔다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S36" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </ns0:c>
       <ns0:c r="F37" t="inlineStr">
         <ns0:is>
-          <ns0:t>북미와 독일에서 상업·산업·정부용 에너지 관리 시스템을 연구·설계·제조·판매·설치한다.</ns0:t>
+          <ns0:t>북미·독일에서 상업·산업·정부용 에너지 관리 시스템을 연구·설계·제조·판매·설치한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G37">
@@ -3056,7 +3056,7 @@
       </ns0:c>
       <ns0:c r="R37" t="inlineStr">
         <ns0:is>
-          <ns0:t>실적 전망 상향과 소매업체 대상 사업 기회의 확실성을 점검하는 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>실적 전망 상향과 소매업체 관련 사업 기회의 확실성을 점검한 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S37" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </ns0:c>
       <ns0:c r="F38" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 유럽에서 금형 성형, CNC 가공, 3D 프린팅, 판금 등 맞춤형 부품 제조 서비스를 제공한다.</ns0:t>
+          <ns0:t>미국·유럽에서 금형 성형, CNC 가공, 3D 프린팅, 판금 등 맞춤형 부품 제조 서비스를 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G38">
@@ -3140,7 +3140,7 @@
       </ns0:c>
       <ns0:c r="R38" t="inlineStr">
         <ns0:is>
-          <ns0:t>매도를 주장하는 근거와 향후 사업 전개에 숨은 위험을 짚는 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>매도 근거를 제시하는 기사와 향후 사업 전개에 숨은 위험을 묻는 기사가 나왔다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S38" t="inlineStr">
@@ -3182,7 +3182,7 @@
       </ns0:c>
       <ns0:c r="F39" t="inlineStr">
         <ns0:is>
-          <ns0:t>바이오 공정 기술과 시스템을 개발·상용화하며 중공사 소모품, 크로마토그래피 시스템 등을 제공한다.</ns0:t>
+          <ns0:t>바이오 공정 기술·시스템을 개발·상용화하며 중공사 소모품과 크로마토그래피 시스템 등을 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G39">
@@ -3224,7 +3224,7 @@
       </ns0:c>
       <ns0:c r="R39" t="inlineStr">
         <ns0:is>
-          <ns0:t>투자 회피 근거를 제시하는 의견과 최근 반등 후 적정 가치에 근접했다는 평가. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>투자 회피 근거를 제시하는 기사와 최근 반등 후 주가가 적정 가치에 근접했다는 평가가 나왔다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S39" t="inlineStr">
@@ -3266,7 +3266,7 @@
       </ns0:c>
       <ns0:c r="F40" t="inlineStr">
         <ns0:is>
-          <ns0:t>암호화폐 채굴용 액체냉각 기술을 개발하며, 비트코인 채굴기 냉각 전환 캐비닛과 실외 인프라 제품을 제공.</ns0:t>
+          <ns0:t>암호화폐 채굴용 액체냉각 기술과 비트코인 채굴기 냉각 전환 캐비닛·실외 인프라 제품을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G40">
@@ -3345,7 +3345,7 @@
       </ns0:c>
       <ns0:c r="F41" t="inlineStr">
         <ns0:is>
-          <ns0:t>주로 오하이오의 개인·기업에 상업은행·신탁·자산관리·권원보험을 제공하는 State Bank and Trust의 지주사.</ns0:t>
+          <ns0:t>오하이오 개인·기업에 은행·신탁·자산관리·권원보험을 제공하는 State Bank and Trust의 지주사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G41">
@@ -3387,7 +3387,7 @@
       </ns0:c>
       <ns0:c r="R41" t="inlineStr">
         <ns0:is>
-          <ns0:t>투자 매력과 저평가 여부, 주가 신고점 이후 추가 상승 여력을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>투자 매력과 저평가 여부, 신고가 기록 이후 추가 상승 여력을 살펴보는 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S41" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </ns0:c>
       <ns0:c r="F42" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 주요 안질환 치료를 위한 수술·비수술 기술을 개발하고 상용화하는 안과 의료기기 기업이다.</ns0:t>
+          <ns0:t>미국에서 주요 안질환 치료용 수술·비수술 기술을 개발·상용화하는 안과 의료기기 기업이다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G42">
@@ -3587,7 +3587,7 @@
       </ns0:c>
       <ns0:c r="F44" t="inlineStr">
         <ns0:is>
-          <ns0:t>치료제, 진단, 화학·소재, 식품·농업, 데이터 저장과 학술 연구에 쓰이는 합성 DNA 제품을 제조·판매한다.</ns0:t>
+          <ns0:t>치료제·진단·화학·소재·식품·농업·데이터 저장·학술 연구용 합성 DNA 제품을 제조·판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G44">
@@ -3629,7 +3629,7 @@
       </ns0:c>
       <ns0:c r="R44" t="inlineStr">
         <ns0:is>
-          <ns0:t>투자 판단 조건, 급등과 앤트로픽의 연관성에 대한 리링크의 해석, 릴리 TuneLab과의 AI 신약 개발 협력을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>매수 판단 조건, 주가 급등과 앤트로픽의 연관성에 대한 리링크의 해석, 릴리 TuneLab 협력을 다뤘다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S44" t="inlineStr">
@@ -3671,7 +3671,7 @@
       </ns0:c>
       <ns0:c r="F45" t="inlineStr">
         <ns0:is>
-          <ns0:t>생물학적 시스템 분석용 장비, 소모품, 소프트웨어를 개발·판매하며 Chromium 플랫폼을 제공한다.</ns0:t>
+          <ns0:t>생물학적 시스템 분석용 장비·소모품·소프트웨어를 개발·판매하며 Chromium 플랫폼을 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G45">
@@ -3713,7 +3713,7 @@
       </ns0:c>
       <ns0:c r="R45" t="inlineStr">
         <ns0:is>
-          <ns0:t>의료·생명과학 종목들과 동반 하락한 흐름 및 동종 기업 대비 2분기 실적을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>의료 관련 종목들과 동반 하락한 소식과 생명과학 도구·서비스 기업 간 2분기 실적 비교를 다뤘다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S45" t="inlineStr">
@@ -3831,7 +3831,7 @@
       </ns0:c>
       <ns0:c r="F47" t="inlineStr">
         <ns0:is>
-          <ns0:t>분석 업무 솔루션을 제공하며 액체 크로마토그래피와 질량분석 시스템을 설계·제조·판매·서비스한다.</ns0:t>
+          <ns0:t>분석 업무 솔루션을 제공하며 액체 크로마토그래피·질량분석 시스템을 설계·제조·판매·서비스한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G47">
@@ -3873,7 +3873,7 @@
       </ns0:c>
       <ns0:c r="R47" t="inlineStr">
         <ns0:is>
-          <ns0:t>가정용 HPV 검사·세포 분석 확대, AI 수요와 BD 통합을 배경으로 한 성장 전망 상회, 견조한 실적을 다룬 기사. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>가정용 HPV·세포 분석 사업, AI 수요·BD 통합 관련 성장 전망 상회, 견조한 실적을 다뤘다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S47" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </ns0:c>
       <ns0:c r="F48" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술 서비스 분야 기업과 합병, 주식 교환, 자산 인수, 자본 재편 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>기술 서비스 기업과 합병, 주식 교환, 자산 인수, 자본 재편 등 기업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G48">
@@ -3957,7 +3957,7 @@
       </ns0:c>
       <ns0:c r="R48" t="inlineStr">
         <ns0:is>
-          <ns0:t>에버노스의 XRP 재무자산 보유 종목 XRPN이 나스닥 진출까지 표결 하나를 남겨뒀다는 보도. (기사 제목 요약·주가 인과 미확정)</ns0:t>
+          <ns0:t>에버노스의 XRP 재무자산 보유 주식 XRPN이 나스닥 진출까지 표결 한 차례를 남겼다는 기사다. (기사 제목 요약·주가 인과 미확정)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S48" t="inlineStr">

</xml_diff>